<commit_message>
docs(arquitectura): se agregan diagramas de clases, secuencia y modelo de datos (DER)
</commit_message>
<xml_diff>
--- a/Plan Entrega IS y TD 2026.xlsx
+++ b/Plan Entrega IS y TD 2026.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBBCD75F-BCD7-4222-817D-9DF17317DF92}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="699" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28905" yWindow="60" windowWidth="14610" windowHeight="15585" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -61,9 +61,6 @@
     <t>T02. Gestión de Login/Logout y gestión de usuarios</t>
   </si>
   <si>
-    <t>Análisis, diseño e implementación. Se espera la utilización del patrón Singleton. Permite verificar la identidad del usuario a través del ingreso de su nombre de usuario y su clave, asignándole el perfil que tenga asignado en el sistema. Se debe describir como será la política de ‘log-in’ / ‘log-out‘. También deberán diferenciarse y documentarse los procesos que se correrán en el arranque del sistema, el log in, y el apagado de sistema, el log-out (permisos, audioria, control de integridad, etc). .  Deberá considerar los siguientes items: Objetivo, Descripción detallada de cómo funciona, Diagrama de clases, DER (Si es necesario), Secuencia (Si es necesario) y el diseño de los algoritmos que sean necesarios. Se espera el uso del patrón singleton.</t>
-  </si>
-  <si>
     <t>documentación - implementación - patrón singleton</t>
   </si>
   <si>
@@ -362,12 +359,97 @@
   <si>
     <t>Planificación TD  - 2026</t>
   </si>
+  <si>
+    <r>
+      <t>Análisis, diseño e implementación. Se espera la utilización del patrón Singleton. Permite verificar la identidad del usuario a través del ingreso de su nombre de usuario y su clave, asignándole el perfil que tenga asignado en el sistema. Se debe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>describir como será la política de ‘log-in’ / ‘log-out‘</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. También deberán diferenciarse y </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>documentarse los procesos que se correrán en el arranque del sistema, el log in, y el apagado de sistema, el log-out (permisos, audioria, control de integridad, etc). .</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  Deberá considerar los siguientes items</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Objetivo, Descripción detallada de cómo funciona</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Diagrama de clases, DER (Si es necesario), Secuencia (Si es necesario) y el diseño de los algoritmos que sean necesarios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Se espera el uso del patrón singleton.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,6 +461,26 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -872,7 +974,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -974,27 +1076,51 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1004,35 +1130,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1347,13 +1452,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
-        <v>100</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
+      <c r="A1" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1373,14 +1478,14 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="51">
+      <c r="A3" s="48">
         <v>1</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="61" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="18" t="s">
@@ -1388,206 +1493,206 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51"/>
+      <c r="A4" s="48"/>
       <c r="B4" s="19"/>
       <c r="C4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="E4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="18" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="51"/>
+      <c r="A5" s="48"/>
       <c r="B5" s="19"/>
       <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="51"/>
+      <c r="A6" s="48"/>
       <c r="B6" s="19"/>
       <c r="C6" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="E6" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="18" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56">
+      <c r="A7" s="53">
         <v>2</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>18</v>
-      </c>
       <c r="E7" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="270.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="57"/>
+      <c r="A8" s="54"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>20</v>
-      </c>
       <c r="E8" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="57"/>
+      <c r="A9" s="54"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="E9" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>23</v>
-      </c>
     </row>
     <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="57"/>
+      <c r="A10" s="54"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" s="18"/>
     </row>
     <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
+      <c r="A11" s="55"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>27</v>
-      </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="52">
+      <c r="A12" s="47">
         <v>3</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="51"/>
+      <c r="A13" s="48"/>
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="51"/>
+      <c r="A14" s="48"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="51"/>
+      <c r="A15" s="48"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="E15" s="18" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="53"/>
+      <c r="A16" s="52"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="E16" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="18" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="49" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
     </row>
     <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>1</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="56" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="57"/>
+      <c r="D18" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="C18" s="49"/>
-      <c r="D18" s="5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
         <v>2</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="60"/>
+      <c r="D19" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="C19" s="55"/>
-      <c r="D19" s="6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -1595,11 +1700,11 @@
         <v>3</v>
       </c>
       <c r="B20" s="44" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="58"/>
+      <c r="D20" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="C20" s="50"/>
-      <c r="D20" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1607,11 +1712,11 @@
         <v>4</v>
       </c>
       <c r="B21" s="43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" s="44"/>
       <c r="D21" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1619,11 +1724,11 @@
         <v>5</v>
       </c>
       <c r="B22" s="43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1631,11 +1736,11 @@
         <v>6</v>
       </c>
       <c r="B23" s="43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" s="44"/>
       <c r="D23" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -1643,11 +1748,11 @@
         <v>6</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C24" s="22"/>
       <c r="D24" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1655,11 +1760,11 @@
         <v>7</v>
       </c>
       <c r="B25" s="43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C25" s="44"/>
       <c r="D25" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1667,23 +1772,23 @@
         <v>8</v>
       </c>
       <c r="B26" s="43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C26" s="44"/>
       <c r="D26" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12">
         <v>9</v>
       </c>
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="42"/>
+      <c r="D27" s="8" t="s">
         <v>55</v>
-      </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="8" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1720,17 +1825,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
-        <v>104</v>
-      </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
+      <c r="A1" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -1751,263 +1856,263 @@
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="18" t="s">
-        <v>60</v>
-      </c>
     </row>
     <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="56">
+      <c r="A4" s="53">
         <v>1</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D4" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>62</v>
-      </c>
       <c r="E4" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="57"/>
+      <c r="A5" s="54"/>
       <c r="B5" s="31"/>
       <c r="C5" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>64</v>
-      </c>
       <c r="E5" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="57"/>
+      <c r="A6" s="54"/>
       <c r="B6" s="40"/>
       <c r="C6" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>66</v>
-      </c>
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="57"/>
+      <c r="A7" s="54"/>
       <c r="B7" s="32"/>
       <c r="C7" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="21" t="s">
-        <v>68</v>
-      </c>
       <c r="E7" s="21"/>
     </row>
     <row r="8" spans="1:5" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="57"/>
+      <c r="A8" s="54"/>
       <c r="B8" s="33"/>
       <c r="C8" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="D8" s="25" t="s">
-        <v>70</v>
-      </c>
       <c r="E8" s="25"/>
     </row>
     <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="57"/>
+      <c r="A9" s="54"/>
       <c r="B9" s="34"/>
       <c r="C9" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="21" t="s">
-        <v>72</v>
-      </c>
       <c r="E9" s="21"/>
     </row>
     <row r="10" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="58"/>
+      <c r="A10" s="55"/>
       <c r="B10" s="31"/>
       <c r="C10" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="E10" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="E10" s="18" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="11" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="52">
+      <c r="A11" s="47">
         <v>2</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="E11" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>103</v>
-      </c>
     </row>
     <row r="12" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="53"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="E12" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="18" t="s">
-        <v>79</v>
-      </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="52">
+      <c r="A13" s="47">
         <v>3</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>82</v>
-      </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="51"/>
+      <c r="A14" s="48"/>
       <c r="B14" s="36"/>
       <c r="C14" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="18" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="51"/>
+      <c r="A15" s="48"/>
       <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>87</v>
-      </c>
       <c r="E15" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51"/>
+      <c r="A16" s="48"/>
       <c r="B16" s="37"/>
       <c r="C16" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>89</v>
-      </c>
       <c r="E16" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="51"/>
+      <c r="A17" s="48"/>
       <c r="B17" s="37"/>
       <c r="C17" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="E17" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="51"/>
+      <c r="A18" s="48"/>
       <c r="B18" s="37"/>
       <c r="C18" s="26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>91</v>
-      </c>
       <c r="E18" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="51"/>
+      <c r="A19" s="48"/>
       <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>93</v>
-      </c>
       <c r="E19" s="18"/>
     </row>
     <row r="20" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="51"/>
+      <c r="A20" s="48"/>
       <c r="B20" s="37"/>
       <c r="C20" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D20" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>95</v>
-      </c>
     </row>
     <row r="21" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="51"/>
+      <c r="A21" s="48"/>
       <c r="B21" s="38"/>
       <c r="C21" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="E21" s="18" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="49" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="47" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>1</v>
       </c>
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="50" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="51"/>
+      <c r="D23" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C23" s="60"/>
-      <c r="D23" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -2015,11 +2120,11 @@
         <v>2</v>
       </c>
       <c r="B24" s="43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C24" s="44"/>
       <c r="D24" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -2027,11 +2132,11 @@
         <v>3</v>
       </c>
       <c r="B25" s="43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C25" s="44"/>
       <c r="D25" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2039,11 +2144,11 @@
         <v>4</v>
       </c>
       <c r="B26" s="43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C26" s="44"/>
       <c r="D26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -2051,11 +2156,11 @@
         <v>5</v>
       </c>
       <c r="B27" s="43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C27" s="44"/>
       <c r="D27" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
@@ -2063,11 +2168,11 @@
         <v>6</v>
       </c>
       <c r="B28" s="43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C28" s="44"/>
       <c r="D28" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
@@ -2075,27 +2180,33 @@
         <v>7</v>
       </c>
       <c r="B29" s="43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C29" s="44"/>
       <c r="D29" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12">
         <v>8</v>
       </c>
-      <c r="B30" s="45" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="46"/>
+      <c r="B30" s="41" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="42"/>
       <c r="D30" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A4:A10"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
@@ -2103,12 +2214,6 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A4:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix: Corregir filtro de fecha desde - hasta cuando es el mismo dia.
Feat: Agregar DVH a la tabla de usuario
</commit_message>
<xml_diff>
--- a/Plan Entrega IS y TD 2026.xlsx
+++ b/Plan Entrega IS y TD 2026.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBBCD75F-BCD7-4222-817D-9DF17317DF92}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="60" windowWidth="14610" windowHeight="15585" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -1076,68 +1076,68 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1154,6 +1154,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1444,23 +1448,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.7109375" customWidth="1"/>
-    <col min="5" max="5" width="66.28515625" style="17" customWidth="1"/>
+    <col min="3" max="3" width="64.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="103.7265625" customWidth="1"/>
+    <col min="5" max="5" width="66.26953125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="42" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1477,23 +1481,23 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="48">
+    <row r="3" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="52">
         <v>1</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="61" t="s">
+      <c r="D3" s="41" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="18" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="48"/>
+    <row r="4" spans="1:5" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="52"/>
       <c r="B4" s="19"/>
       <c r="C4" s="18" t="s">
         <v>8</v>
@@ -1505,8 +1509,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="48"/>
+    <row r="5" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="52"/>
       <c r="B5" s="19"/>
       <c r="C5" s="3" t="s">
         <v>10</v>
@@ -1518,8 +1522,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="48"/>
+    <row r="6" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="52"/>
       <c r="B6" s="19"/>
       <c r="C6" s="18" t="s">
         <v>13</v>
@@ -1531,8 +1535,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="53">
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="57">
         <v>2</v>
       </c>
       <c r="B7" s="19"/>
@@ -1546,8 +1550,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="270.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
+    <row r="8" spans="1:5" ht="247" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="58"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>18</v>
@@ -1559,8 +1563,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="54"/>
+    <row r="9" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="58"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
         <v>20</v>
@@ -1572,8 +1576,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="54"/>
+    <row r="10" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="58"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
         <v>23</v>
@@ -1583,8 +1587,8 @@
       </c>
       <c r="E10" s="18"/>
     </row>
-    <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="55"/>
+    <row r="11" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="59"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
         <v>24</v>
@@ -1596,8 +1600,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="47">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="53">
         <v>3</v>
       </c>
       <c r="B12" s="19"/>
@@ -1611,8 +1615,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="48"/>
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="52"/>
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
         <v>28</v>
@@ -1624,8 +1628,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="48"/>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="52"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
         <v>24</v>
@@ -1637,8 +1641,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="48"/>
+    <row r="15" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="52"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
         <v>29</v>
@@ -1650,8 +1654,8 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52"/>
+    <row r="16" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="54"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
         <v>32</v>
@@ -1663,87 +1667,87 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="49" t="s">
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="49"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-    </row>
-    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+    </row>
+    <row r="18" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <v>1</v>
       </c>
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="57"/>
+      <c r="C18" s="50"/>
       <c r="D18" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
         <v>2</v>
       </c>
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="55" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="60"/>
+      <c r="C19" s="56"/>
       <c r="D19" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="11">
         <v>3</v>
       </c>
-      <c r="B20" s="44" t="s">
+      <c r="B20" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="58"/>
+      <c r="C20" s="51"/>
       <c r="D20" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="11">
         <v>4</v>
       </c>
-      <c r="B21" s="43" t="s">
+      <c r="B21" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="44"/>
+      <c r="C21" s="45"/>
       <c r="D21" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="11">
         <v>5</v>
       </c>
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="44"/>
+      <c r="C22" s="45"/>
       <c r="D22" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
         <v>6</v>
       </c>
-      <c r="B23" s="43" t="s">
+      <c r="B23" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="44"/>
+      <c r="C23" s="45"/>
       <c r="D23" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
         <v>6</v>
       </c>
@@ -1755,38 +1759,38 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
         <v>7</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="44"/>
+      <c r="C25" s="45"/>
       <c r="D25" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
         <v>8</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="44"/>
+      <c r="C26" s="45"/>
       <c r="D26" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="12">
         <v>9</v>
       </c>
-      <c r="B27" s="41" t="s">
+      <c r="B27" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="42"/>
+      <c r="C27" s="47"/>
       <c r="D27" s="8" t="s">
         <v>55</v>
       </c>
@@ -1816,24 +1820,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07CA6276-71FC-4BB7-B5A8-70E7B7E3AFEC}">
   <dimension ref="A1:E30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="16"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="4" width="96.28515625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="62.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" style="16"/>
+    <col min="3" max="3" width="67.453125" customWidth="1"/>
+    <col min="4" max="4" width="96.26953125" style="14" customWidth="1"/>
+    <col min="5" max="5" width="62.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="42" t="s">
         <v>103</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="15" t="s">
         <v>56</v>
       </c>
@@ -1850,7 +1854,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="39">
         <v>0</v>
       </c>
@@ -1865,8 +1869,8 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="53">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="57">
         <v>1</v>
       </c>
       <c r="B4" s="31"/>
@@ -1880,8 +1884,8 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="54"/>
+    <row r="5" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="58"/>
       <c r="B5" s="31"/>
       <c r="C5" s="18" t="s">
         <v>62</v>
@@ -1893,8 +1897,8 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="54"/>
+    <row r="6" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="58"/>
       <c r="B6" s="40"/>
       <c r="C6" s="18" t="s">
         <v>64</v>
@@ -1904,8 +1908,8 @@
       </c>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="54"/>
+    <row r="7" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="58"/>
       <c r="B7" s="32"/>
       <c r="C7" s="18" t="s">
         <v>66</v>
@@ -1915,8 +1919,8 @@
       </c>
       <c r="E7" s="21"/>
     </row>
-    <row r="8" spans="1:5" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
+    <row r="8" spans="1:5" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="58"/>
       <c r="B8" s="33"/>
       <c r="C8" s="24" t="s">
         <v>68</v>
@@ -1926,8 +1930,8 @@
       </c>
       <c r="E8" s="25"/>
     </row>
-    <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="54"/>
+    <row r="9" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="58"/>
       <c r="B9" s="34"/>
       <c r="C9" s="18" t="s">
         <v>70</v>
@@ -1937,8 +1941,8 @@
       </c>
       <c r="E9" s="21"/>
     </row>
-    <row r="10" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="55"/>
+    <row r="10" spans="1:5" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="59"/>
       <c r="B10" s="31"/>
       <c r="C10" s="30" t="s">
         <v>72</v>
@@ -1950,8 +1954,8 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="47">
+    <row r="11" spans="1:5" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="53">
         <v>2</v>
       </c>
       <c r="B11" s="19"/>
@@ -1965,8 +1969,8 @@
         <v>102</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="52"/>
+    <row r="12" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="54"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
         <v>76</v>
@@ -1978,8 +1982,8 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="47">
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="53">
         <v>3</v>
       </c>
       <c r="B13" s="35"/>
@@ -1993,8 +1997,8 @@
         <v>81</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="48"/>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="52"/>
       <c r="B14" s="36"/>
       <c r="C14" s="28" t="s">
         <v>82</v>
@@ -2006,8 +2010,8 @@
         <v>84</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="48"/>
+    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="52"/>
       <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
         <v>85</v>
@@ -2019,8 +2023,8 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="48"/>
+    <row r="16" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="52"/>
       <c r="B16" s="37"/>
       <c r="C16" s="26" t="s">
         <v>87</v>
@@ -2032,8 +2036,8 @@
         <v>84</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="48"/>
+    <row r="17" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="52"/>
       <c r="B17" s="37"/>
       <c r="C17" s="29" t="s">
         <v>76</v>
@@ -2045,8 +2049,8 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="48"/>
+    <row r="18" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="52"/>
       <c r="B18" s="37"/>
       <c r="C18" s="26" t="s">
         <v>89</v>
@@ -2058,8 +2062,8 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="48"/>
+    <row r="19" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="52"/>
       <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
         <v>91</v>
@@ -2069,8 +2073,8 @@
       </c>
       <c r="E19" s="18"/>
     </row>
-    <row r="20" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="48"/>
+    <row r="20" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="52"/>
       <c r="B20" s="37"/>
       <c r="C20" s="18" t="s">
         <v>93</v>
@@ -2082,8 +2086,8 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="48"/>
+    <row r="21" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="52"/>
       <c r="B21" s="38"/>
       <c r="C21" s="18" t="s">
         <v>95</v>
@@ -2095,118 +2099,112 @@
         <v>96</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="49" t="s">
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="48" t="s">
         <v>97</v>
       </c>
-      <c r="B22" s="49"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="49"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9">
         <v>1</v>
       </c>
-      <c r="B23" s="50" t="s">
+      <c r="B23" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="51"/>
+      <c r="C23" s="61"/>
       <c r="D23" s="5" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="11">
         <v>2</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="44"/>
+      <c r="C24" s="45"/>
       <c r="D24" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
         <v>3</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="44"/>
+      <c r="C25" s="45"/>
       <c r="D25" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="11">
         <v>4</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="44"/>
+      <c r="C26" s="45"/>
       <c r="D26" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
         <v>5</v>
       </c>
-      <c r="B27" s="43" t="s">
+      <c r="B27" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="44"/>
+      <c r="C27" s="45"/>
       <c r="D27" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="11">
         <v>6</v>
       </c>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="C28" s="44"/>
+      <c r="C28" s="45"/>
       <c r="D28" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
         <v>7</v>
       </c>
-      <c r="B29" s="43" t="s">
+      <c r="B29" s="44" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="44"/>
+      <c r="C29" s="45"/>
       <c r="D29" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="12">
         <v>8</v>
       </c>
-      <c r="B30" s="41" t="s">
+      <c r="B30" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="42"/>
+      <c r="C30" s="47"/>
       <c r="D30" s="8" t="s">
         <v>98</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A4:A10"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
@@ -2214,6 +2212,12 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A4:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: Agregar digito verificador vertical
</commit_message>
<xml_diff>
--- a/Plan Entrega IS y TD 2026.xlsx
+++ b/Plan Entrega IS y TD 2026.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBBCD75F-BCD7-4222-817D-9DF17317DF92}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B76A365-DC9E-4ABA-9C18-5B5F60CBD309}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28905" yWindow="60" windowWidth="14610" windowHeight="15585" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -89,9 +89,6 @@
   </si>
   <si>
     <t>T07. Gestión de DV</t>
-  </si>
-  <si>
-    <t>Análisis, diseño e implementación. La función de los dígitos verificadores es la de permitir comprobar la integridad de los datos almacenados en la base de datos. Se desea poder detectar dos cosas. La primera es si se han agregado o quitado datos de la base de datos por fuera del sistema y la segunda es si se han intercambiado datos de posición. Para esto último es importante, al momento de determinar el algoritmo de cálculo a emplear, que en el cálculo no sólo participe el contenido del atributo sino también la posición del carácter y la posición del atributo dentro de la entidad. Al iniciar la aplicación, y antes de dar acceso a la ventana de log-in, se debe realizar el proceso de verificación de integridad de la base de datos. En caso de error, se deberá informar al administrador para que tome las medidas adecuadas. Los dígitos verificadores horizontales se guardan en un atributo de las entidades bajo análisis mientras que los verticales se pueden guardar en una entidad adicional creada para ese fin, la cual deberá formar parte del DER. Se espera que la verificación de integridad se realice en al menios una entidad de negocio, siendo esta la  más sensible y relevante del sistema. Cuando se desarrolle la especificación correspondiente a esta funcionalidad se deberá contemplar: Detalle de cómo se utilizarán los dígitos verificadores horizontal y vertical. Descripción de las operaciones de restauración a realizar en caso de error en alguno de ellos. Algoritmo a implementar para los cálculos. SE valorará el diseño de un mecanismo genérico para que sea aplicable a cualquier entidad. Deberá considerar los siguientes items: Objetivo, Descripción detallada de cómo funciona, Diagrama de clases, DER (Si es necesario), Secuencia (Si es necesario) y el diseño de los algoritmos que sean necesarios. En caso de que el estado de un objeto se proviene de varias tablas, deberá proponer una solución al problema de la integridad.</t>
   </si>
   <si>
     <t>T04. Gestión de Perfiles de Usuario</t>
@@ -444,6 +441,71 @@
       <t>. Se espera el uso del patrón singleton.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Análisis, diseño e implementación. La función de los dígitos verificadores es la de permitir comprobar la integridad de los datos almacenados en la base de datos. Se desea poder detectar dos cosas. La primera es si se han agregado o quitado datos de la base de datos por fuera del sistema y la segunda es si se han intercambiado datos de posición. Para esto último es importante, al momento de determinar el algoritmo de cálculo a emplear, que en el cálculo no sólo participe el contenido del atributo sino también la posición del carácter y la posición del atributo dentro de la entidad. Al iniciar la aplicación, y antes de dar acceso a la ventana de log-in, se debe realizar el proceso de verificación de integridad de la base de datos. En caso de error, se deberá informar al administrador para que tome las medidas adecuadas. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Los dígitos verificadores horizontales se guardan en un atributo de las entidades bajo análisis mientras que los verticales se pueden guardar en una entidad adicional creada para ese fin, la cual deberá formar parte del DER.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Se espera que la verificación de integridad se realice </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>en al menios una entidad de negocio</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, siendo esta la  más sensible y relevante del sistema. Cuando se desarrolle la especificación correspondiente a esta funcionalidad se deberá contemplar: Detalle de cómo se utilizarán los dígitos verificadores horizontal y vertical. Descripción de las operaciones de restauración a realizar en caso de error en alguno de ellos. Algoritmo a implementar para los cálculos. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SE valorará el diseño de un mecanismo genérico para que sea aplicable a cualquier entidad.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Deberá considerar los siguientes items: Objetivo, Descripción detallada de cómo funciona, Diagrama de clases, DER (Si es necesario), Secuencia (Si es necesario) y el diseño de los algoritmos que sean necesarios. En caso de que el estado de un objeto se proviene de varias tablas, deberá proponer una solución al problema de la integridad.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1154,10 +1216,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1448,23 +1506,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="64.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.7265625" customWidth="1"/>
-    <col min="5" max="5" width="66.26953125" style="17" customWidth="1"/>
+    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="116.85546875" customWidth="1"/>
+    <col min="5" max="5" width="66.28515625" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="42" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
       <c r="D1" s="43"/>
       <c r="E1" s="43"/>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1481,7 +1539,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="52">
         <v>1</v>
       </c>
@@ -1496,20 +1554,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="52"/>
       <c r="B4" s="19"/>
       <c r="C4" s="18" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E4" s="18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="52"/>
       <c r="B5" s="19"/>
       <c r="C5" s="3" t="s">
@@ -1522,7 +1580,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52"/>
       <c r="B6" s="19"/>
       <c r="C6" s="18" t="s">
@@ -1535,7 +1593,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="57">
         <v>2</v>
       </c>
@@ -1550,76 +1608,76 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="247" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="240.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="58"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>19</v>
+        <v>104</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="58"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="E9" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="58"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E10" s="18"/>
     </row>
-    <row r="11" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="59"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="E11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="53">
         <v>3</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="52"/>
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>17</v>
@@ -1628,171 +1686,171 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="52"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>17</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="52"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="21" t="s">
+      <c r="E15" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="18" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="E16" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="18" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="48" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="48" t="s">
-        <v>35</v>
       </c>
       <c r="B17" s="48"/>
       <c r="C17" s="48"/>
       <c r="D17" s="48"/>
     </row>
-    <row r="18" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>1</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C18" s="50"/>
       <c r="D18" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="10">
         <v>2</v>
       </c>
       <c r="B19" s="55" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C19" s="56"/>
       <c r="D19" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>3</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="51"/>
       <c r="D20" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
         <v>4</v>
       </c>
       <c r="B21" s="44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="45"/>
       <c r="D21" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>5</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
         <v>6</v>
       </c>
       <c r="B23" s="44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="45"/>
       <c r="D23" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>6</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="22"/>
       <c r="D24" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>7</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>8</v>
       </c>
       <c r="B26" s="44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12">
         <v>9</v>
       </c>
       <c r="B27" s="46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C27" s="47"/>
       <c r="D27" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1820,26 +1878,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07CA6276-71FC-4BB7-B5A8-70E7B7E3AFEC}">
   <dimension ref="A1:E30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.54296875" style="16"/>
-    <col min="3" max="3" width="67.453125" customWidth="1"/>
-    <col min="4" max="4" width="96.26953125" style="14" customWidth="1"/>
-    <col min="5" max="5" width="62.81640625" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="16"/>
+    <col min="3" max="3" width="67.42578125" customWidth="1"/>
+    <col min="4" max="4" width="96.28515625" style="14" customWidth="1"/>
+    <col min="5" max="5" width="62.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="42" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B1" s="43"/>
       <c r="C1" s="43"/>
       <c r="D1" s="43"/>
       <c r="E1" s="43"/>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
@@ -1854,357 +1912,363 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="39">
         <v>0</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="57">
         <v>1</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="D4" s="20" t="s">
-        <v>61</v>
-      </c>
       <c r="E4" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="58"/>
       <c r="B5" s="31"/>
       <c r="C5" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>63</v>
-      </c>
       <c r="E5" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="58"/>
       <c r="B6" s="40"/>
       <c r="C6" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>65</v>
-      </c>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="58"/>
       <c r="B7" s="32"/>
       <c r="C7" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="21" t="s">
-        <v>67</v>
-      </c>
       <c r="E7" s="21"/>
     </row>
-    <row r="8" spans="1:5" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:5" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="58"/>
       <c r="B8" s="33"/>
       <c r="C8" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="25" t="s">
-        <v>69</v>
-      </c>
       <c r="E8" s="25"/>
     </row>
-    <row r="9" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="58"/>
       <c r="B9" s="34"/>
       <c r="C9" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="21" t="s">
-        <v>71</v>
-      </c>
       <c r="E9" s="21"/>
     </row>
-    <row r="10" spans="1:5" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
       <c r="B10" s="31"/>
       <c r="C10" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="E10" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="E10" s="18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="44" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>2</v>
       </c>
       <c r="B11" s="19"/>
       <c r="C11" s="30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="54"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="E12" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>3</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="52"/>
       <c r="B14" s="36"/>
       <c r="C14" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E14" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="E14" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="52"/>
       <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>86</v>
-      </c>
       <c r="E15" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="52"/>
       <c r="B16" s="37"/>
       <c r="C16" s="26" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>88</v>
-      </c>
       <c r="E16" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="52"/>
       <c r="B17" s="37"/>
       <c r="C17" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>77</v>
-      </c>
       <c r="E17" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="52"/>
       <c r="B18" s="37"/>
       <c r="C18" s="26" t="s">
+        <v>88</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="E18" s="18" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="52"/>
       <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>92</v>
-      </c>
       <c r="E19" s="18"/>
     </row>
-    <row r="20" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="52"/>
       <c r="B20" s="37"/>
       <c r="C20" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="D20" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="21" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="52"/>
       <c r="B21" s="38"/>
       <c r="C21" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="D21" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="18" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="48" t="s">
         <v>96</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="48" t="s">
-        <v>97</v>
       </c>
       <c r="B22" s="48"/>
       <c r="C22" s="48"/>
       <c r="D22" s="48"/>
     </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>1</v>
       </c>
       <c r="B23" s="60" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="61"/>
       <c r="D23" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>2</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>3</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="45"/>
       <c r="D25" s="7" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>4</v>
       </c>
       <c r="B26" s="44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C26" s="45"/>
       <c r="D26" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
         <v>5</v>
       </c>
       <c r="B27" s="44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C27" s="45"/>
       <c r="D27" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
         <v>6</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
         <v>7</v>
       </c>
       <c r="B29" s="44" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" s="45"/>
       <c r="D29" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12">
         <v>8</v>
       </c>
       <c r="B30" s="46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C30" s="47"/>
       <c r="D30" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A4:A10"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
@@ -2212,12 +2276,6 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A4:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix: Recursividad en Roles y Permisos
</commit_message>
<xml_diff>
--- a/Plan Entrega IS y TD 2026.xlsx
+++ b/Plan Entrega IS y TD 2026.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B76A365-DC9E-4ABA-9C18-5B5F60CBD309}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10B3FBA3-3B92-42B7-BDD0-22C16FEF2DE7}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="60" windowWidth="14610" windowHeight="15585" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -443,7 +443,49 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Análisis, diseño e implementación. La función de los dígitos verificadores es la de permitir comprobar la integridad de los datos almacenados en la base de datos. Se desea poder detectar dos cosas. La primera es si se han agregado o quitado datos de la base de datos por fuera del sistema y la segunda es si se han intercambiado datos de posición. Para esto último es importante, al momento de determinar el algoritmo de cálculo a emplear, que en el cálculo no sólo participe el contenido del atributo sino también la posición del carácter y la posición del atributo dentro de la entidad. Al iniciar la aplicación, y antes de dar acceso a la ventana de log-in, se debe realizar el proceso de verificación de integridad de la base de datos. En caso de error, se deberá informar al administrador para que tome las medidas adecuadas. </t>
+      <t xml:space="preserve">Análisis, diseño e implementación. La función de los dígitos verificadores es la de permitir comprobar la integridad de los datos almacenados en la base de datos. Se desea poder detectar dos cosas. La primera es </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>si se han agregado o quitado datos de la base de datos por fuera del sistema</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> y la segunda es</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> si se han intercambiado datos de posición</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Para esto último es importante, al momento de determinar el algoritmo de cálculo a emplear, que en el cálculo no sólo participe el contenido del atributo sino también la posición del carácter y la posición del atributo dentro de la entidad. Al iniciar la aplicación, y antes de dar acceso a la ventana de log-in, se debe realizar el proceso de verificación de integridad de la base de datos. En caso de error, se deberá informar al administrador para que tome las medidas adecuadas. </t>
     </r>
     <r>
       <rPr>
@@ -511,7 +553,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -547,6 +589,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1216,6 +1274,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1539,7 +1601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="52">
         <v>1</v>
       </c>
@@ -1554,7 +1616,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="52"/>
       <c r="B4" s="19"/>
       <c r="C4" s="18" t="s">
@@ -1567,7 +1629,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="52"/>
       <c r="B5" s="19"/>
       <c r="C5" s="3" t="s">
@@ -1580,7 +1642,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52"/>
       <c r="B6" s="19"/>
       <c r="C6" s="18" t="s">
@@ -1608,7 +1670,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="240.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="248.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="58"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
@@ -1634,7 +1696,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="58"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
@@ -1712,7 +1774,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="54"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
@@ -1817,7 +1879,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Feat: Agregar solo Rol Admin tiene acceso a frmSeguridad Feat: Agregar un usuario de emergencia si el admin es borrado
</commit_message>
<xml_diff>
--- a/Plan Entrega IS y TD 2026.xlsx
+++ b/Plan Entrega IS y TD 2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10B3FBA3-3B92-42B7-BDD0-22C16FEF2DE7}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14505" yWindow="60" windowWidth="14610" windowHeight="15585" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -1274,10 +1274,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2325,12 +2321,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A4:A10"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
@@ -2338,6 +2328,12 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A4:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>